<commit_message>
Integrate SEG015/016 peripheral makers into deck, xlsx, flow
Regenerate master xlsx (145 companies), add two appendix slides for
semiconductor equipment components/subsystems (SMC, Horiba, Advantest,
Nippon Pillar, Daifuku...) and electronic parts/substrates/gases
(Murata, Ibiden, TDK, Taiyo Yuden, Nippon Sanso...), and note the
downstream spillover on the value-chain flow (deck slide 2 + flow HTML).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017hVm54qQ8iaGNRYcCDuKBy
</commit_message>
<xml_diff>
--- a/output/valuechain_master.xlsx
+++ b/output/valuechain_master.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="valuechain_master" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="segments" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="sources" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="valuechain_master" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="segments" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sources" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P129"/>
+  <dimension ref="A1:P146"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -10346,6 +10346,1366 @@
         </is>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>15</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>SEG015</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>半導体製造装置 部品・サブシステム</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>C144</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>アドバンテスト</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>Advantest Corporation</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>6857</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L130" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M130" t="inlineStr">
+        <is>
+          <t>AI向け高性能半導体（GPU/HBM/SoC）向け半導体テスタ需要の急拡大により2026年3月期は売上高1兆1286億円（+44.7%）・営業利益4991億円（+118.8%）と過去最高を更新し、2027年3月期は売上高1兆4200億円へさらに拡大を計画。</t>
+        </is>
+      </c>
+      <c r="N130" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O130" t="inlineStr">
+        <is>
+          <t>2026年3月期 決算短信〔IFRS〕(連結)（https://www.advantest.com/ja/news/2026/a81o6o0000000heh-att/J_FR_FY2025_FN.pdf）</t>
+        </is>
+      </c>
+      <c r="P130" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>15</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>SEG015</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>半導体製造装置 部品・サブシステム</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>C141</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>イーグル工業</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>Eagle Industry Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>6486</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L131" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M131" t="inlineStr">
+        <is>
+          <t>半導体製造装置向けメカニカルシールが下期以降に生成AI関連分野中心に回復し、2026年3月期は売上高1774.9億円・営業利益134.7億円（+58.6%）で売上高・経常利益とも過去最高。2027年3月期も生成AI普及を背景に半導体向け販売増を見込む。</t>
+        </is>
+      </c>
+      <c r="N131" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O131" t="inlineStr">
+        <is>
+          <t>イーグル工業 決算説明会書き起こし（https://finance.yahoo.co.jp/quote/6486.T/financials?styl=presentation）</t>
+        </is>
+      </c>
+      <c r="P131" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>15</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>SEG015</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>半導体製造装置 部品・サブシステム</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>C145</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>ダイフク</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>Daifuku Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>6383</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L132" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>半導体クリーンルーム向けAMHS（自動搬送システム）で世界大手。生成AIによる先端半導体投資拡大を背景に2026年3月期第1四半期の受注高が2213億円（+54.7%）と過去最高を更新し、売上・営業利益とも増加。</t>
+        </is>
+      </c>
+      <c r="N132" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O132" t="inlineStr">
+        <is>
+          <t>ダイフク【6383】IR情報・決算短信（https://www.nikkei.com/nkd/company/kigyo/?scode=6383）</t>
+        </is>
+      </c>
+      <c r="P132" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>15</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>SEG015</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>半導体製造装置 部品・サブシステム</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>C142</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>堀場製作所</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>HORIBA Ltd.</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>6856</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L133" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>半導体製造装置向けマスフローコントローラ（世界シェア約6割）が主力で、AI・データセンター需要を背景にアジアの半導体装置メーカー向け販売が拡大。半導体セグメントの好調で2026年12月期通期見通しを売上高3730億円・営業利益680億円（+28.2%）へ上方修正。</t>
+        </is>
+      </c>
+      <c r="N133" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O133" t="inlineStr">
+        <is>
+          <t>堀場製作所 2026年12月期 第1四半期決算・通期見通し（https://www.ir-tracker.com/ja/articles/6856-2026-Q1）</t>
+        </is>
+      </c>
+      <c r="P133" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>15</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>SEG015</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>半導体製造装置 部品・サブシステム</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>C140</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>日本ピラー工業</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>Nippon Pillar Packing Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>6490</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L134" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M134" t="inlineStr">
+        <is>
+          <t>半導体向け超純水・薬液用フッ素樹脂継手/メカニカルシールで高シェアを持ち、AI半導体の微細化・洗浄工程増で需要拡大。2026年3月期は売上高594.8億円・営業利益121.1億円と増収増益、2027年3月期は売上高700億円・営業利益155億円へ大幅拡大を計画。</t>
+        </is>
+      </c>
+      <c r="N134" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O134" t="inlineStr">
+        <is>
+          <t>PILLAR【6490】決算発表・業績情報（https://www.nikkei.com/nkd/company/kessan/?scode=6490）</t>
+        </is>
+      </c>
+      <c r="P134" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>15</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>SEG015</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>半導体製造装置 部品・サブシステム</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>C139</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>CKD</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>CKD Corporation</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>6407</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L135" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>空気圧・流体制御機器および半導体製造装置向けコンポーネント（薬液用バルブ等）が主力で、半導体関連需要は堅調に推移し海外向け販売が伸長。全社では自動機械の反動減で2026年3月期は減益だが半導体部品事業はAI投資を追い風に底堅い。</t>
+        </is>
+      </c>
+      <c r="N135" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="O135" t="inlineStr">
+        <is>
+          <t>IR説明会資料・決算資料（https://www.ckd.co.jp/ir/kessan/）</t>
+        </is>
+      </c>
+      <c r="P135" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>15</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>SEG015</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>半導体製造装置 部品・サブシステム</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>C138</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>SMC</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>SMC Corporation</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>6273</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L136" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M136" t="inlineStr">
+        <is>
+          <t>空気圧制御機器の世界トップ（グローバルシェア約4割）として半導体製造装置に多用され、AI半導体の前工程投資回復を背景に2026年3月期は売上高8425億円（+6.4%）・経常利益2356億円（+12.2%）と半導体関連需要回復で増収増益。</t>
+        </is>
+      </c>
+      <c r="N136" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="O136" t="inlineStr">
+        <is>
+          <t>SMC【6273】決算発表・業績情報（https://www.nikkei.com/nkd/company/kessan/?scode=6273）</t>
+        </is>
+      </c>
+      <c r="P136" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>15</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>SEG015</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>半導体製造装置 部品・サブシステム</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>C146</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>フェローテックホールディングス</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>Ferrotec Holdings Corporation</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>6890</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>東証スタンダード</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L137" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>半導体製造装置向け真空シール・石英/セラミック等の部品・消耗品事業が主力で、生成AIサーバー投資・メモリ製造装置投資の拡大が追い風。2026年3月期は半導体等装置関連事業が好調で増収増益、部品加工能力の増強を推進。</t>
+        </is>
+      </c>
+      <c r="N137" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="O137" t="inlineStr">
+        <is>
+          <t>2026年3月期 決算説明資料・中期経営計画骨子（https://japanir.jp/company/company-6890/ir/6890-20260518-01_wp_financial_summary/）</t>
+        </is>
+      </c>
+      <c r="P137" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>15</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>SEG015</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>半導体製造装置 部品・サブシステム</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>C143</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>ローツェ</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>Rorze Corporation</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>6323</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M138" t="inlineStr">
+        <is>
+          <t>半導体搬送ロボット・EFEM・ロードポートで世界シェア25〜35%の隠れたニッチトップ。Applied Materials・TSMCが主要顧客で、AI半導体の前工程装置需要拡大が追い風。2026年2月期は売上高1287.9億円（+3.5%）と増収だが訴訟引当等で減益。</t>
+        </is>
+      </c>
+      <c r="N138" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="O138" t="inlineStr">
+        <is>
+          <t>ローツェ 企業情報・業績（EFEM世界シェア25〜35%）（https://www.buffett-code.com/company/6323/）</t>
+        </is>
+      </c>
+      <c r="P138" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>16</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>SEG016</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>電子部品・パッケージ基板・産業ガス等（周辺・下流）</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>C150</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>TDK</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>TDK Corporation</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>6762</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M139" t="inlineStr">
+        <is>
+          <t>AIデータセンター向けニアラインHDD用部品・パッシブ部品が牽引し2026年3月期は売上高2兆5048億円（+13.6%）・営業利益2724億円（+21.5%）と過去最高。経営陣はAIデータセンター向けパッシブ部品売上を約10倍に拡大する方針を表明。</t>
+        </is>
+      </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O139" t="inlineStr">
+        <is>
+          <t>TDK Posts Record Profits Driven by AI Data Center Demand (FY2026 Full-Year Earnings Call)（https://finance.biggo.com/news/JP_6762.T_2026-04-28）</t>
+        </is>
+      </c>
+      <c r="P139" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>16</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>SEG016</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>電子部品・パッケージ基板・産業ガス等（周辺・下流）</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>C147</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>イビデン</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>Ibiden Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>4062</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M140" t="inlineStr">
+        <is>
+          <t>生成AIサーバー向けICパッケージ基板の受注が堅調で2026年3月期は売上高4162億円（+12.7%）・営業利益620億円（+30.3%）と増収増益。2026年度から3年間で総額5000億円を投じAIサーバー向け基板の生産能力を2028年3月期に2.5倍へ拡大する計画。</t>
+        </is>
+      </c>
+      <c r="N140" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O140" t="inlineStr">
+        <is>
+          <t>イビデン、半導体部品増産へ5000億円投資 生成AIサーバー向け（https://www.nikkei.com/article/DGXZQOFD0370L0T00C26A2000000/）</t>
+        </is>
+      </c>
+      <c r="P140" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>16</v>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>SEG016</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>電子部品・パッケージ基板・産業ガス等（周辺・下流）</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>C153</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>トリケミカル研究所</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>Tri Chemical Laboratories Inc.</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>4369</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M141" t="inlineStr">
+        <is>
+          <t>半導体微細化に不可欠なHigh-k材料等の超高純度前駆体材料で高シェア。生成AI需要を背景に2026年1月期第3四半期累計は売上高180.1億円（+37.4%）・営業利益45.6億円（+30.2%）と増収増益、2027年1月期もAI半導体向け需要増が続く。</t>
+        </is>
+      </c>
+      <c r="N141" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O141" t="inlineStr">
+        <is>
+          <t>トリケミカル研究所（4369）2026年1月期3Q決算：生成AI需要で3割増益（https://note.com/jstock_lab/n/n3d8f9723f4aa）</t>
+        </is>
+      </c>
+      <c r="P141" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>16</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>SEG016</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>電子部品・パッケージ基板・産業ガス等（周辺・下流）</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>C154</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>太陽誘電</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>Taiyo Yuden Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>6976</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M142" t="inlineStr">
+        <is>
+          <t>AIサーバー向けMLCC需要（1台あたり約2.8万個、従来サーバーの約10倍超）が急拡大し2026年3月期は営業利益200億円（+91.2%）・純利益は前年の5.4倍。2027年3月期は営業利益300億円（+50%）を計画し受注のブック・ツー・ビルは1.25と高水準。</t>
+        </is>
+      </c>
+      <c r="N142" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O142" t="inlineStr">
+        <is>
+          <t>太陽誘電、営業益91％増の200億円に急回復 来期は50％増の300億円計画 AIサーバー需要追い風（https://finance.biggo.jp/news/JP_6976.T_2026-05-08）</t>
+        </is>
+      </c>
+      <c r="P142" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>16</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>SEG016</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>電子部品・パッケージ基板・産業ガス等（周辺・下流）</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>C149</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>村田製作所</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>Murata Manufacturing Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>6981</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M143" t="inlineStr">
+        <is>
+          <t>MLCCで世界シェア4割強の首位。AIサーバー1台に約3万個のMLCCが必要（従来サーバーの5〜10倍）で需要が急拡大し、2026年4月から15〜35%の価格改定を実施。2027年3月期はAIサーバー需要を背景に増収・営業利益+34.8%を見込む。</t>
+        </is>
+      </c>
+      <c r="N143" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O143" t="inlineStr">
+        <is>
+          <t>半年で株価3倍の村田製作所、「AIサーバー特需」は続くか（https://toyokeizai.net/articles/-/947755）</t>
+        </is>
+      </c>
+      <c r="P143" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>16</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>SEG016</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>電子部品・パッケージ基板・産業ガス等（周辺・下流）</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>C148</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>新光電気工業</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>Shinko Electric Industries Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>6967</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>非上場（JICによるTOBで上場廃止）</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>非上場</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M144" t="inlineStr">
+        <is>
+          <t>CPU/GPU向け高性能半導体パッケージ基板（FC-BGA）大手で、AI向け半導体需要の拡大がメタルパッケージ事業等を牽引。JIC傘下で非上場化し、AIパッケージング需要を背景に成長投資を進める。</t>
+        </is>
+      </c>
+      <c r="N144" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="O144" t="inlineStr">
+        <is>
+          <t>決算短信 IRライブラリ（https://www.shinko.co.jp/ir/library/summary/）</t>
+        </is>
+      </c>
+      <c r="P144" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>16</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>SEG016</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>電子部品・パッケージ基板・産業ガス等（周辺・下流）</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>C151</t>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>日本酸素ホールディングス</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr">
+        <is>
+          <t>Nippon Sanso Holdings Corporation</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>4091</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr">
+        <is>
+          <t>産業ガス国内首位・エレクトロニクス向け特殊ガスで世界3強。半導体向け特殊ガス・オンサイトガス供給がAI半導体増産を背景に堅調で、2026年3月期第3四半期累計は売上収益9977億円（+2.7%）・営業利益1461億円（+13.5%）と増収増益。</t>
+        </is>
+      </c>
+      <c r="N145" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="O145" t="inlineStr">
+        <is>
+          <t>日本酸素ホールディングス 決算情報（https://finance.matsui.co.jp/stock/4091/settlement/index）</t>
+        </is>
+      </c>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>16</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>SEG016</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>電子部品・パッケージ基板・産業ガス等（周辺・下流）</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>C152</t>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>関東電化工業</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr">
+        <is>
+          <t>Kanto Denka Kogyo Co. Ltd.</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>4047</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr">
+        <is>
+          <t>半導体エッチング・クリーニング用含フッ素特殊ガス等の精密化学品が主力で、AI半導体増産を背景に需要拡大。2026年3月期は売上高654億円（+4.9%）・経常利益66.3億円（+47.1%）と大幅増益、2027年3月期は売上高950億円・経常利益100億円へ拡大を計画。</t>
+        </is>
+      </c>
+      <c r="N146" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="O146" t="inlineStr">
+        <is>
+          <t>関東電化工業 決算発表履歴（適時開示）（https://irbank.net/4047/pl）</t>
+        </is>
+      </c>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10357,7 +11717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10884,6 +12244,76 @@
       <c r="G15" t="inlineStr">
         <is>
           <t>データセンター・工場建設向け資材メーカー</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SEG015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>半導体製造装置 部品・サブシステム</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>15</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>完了</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>流体制御・バルブ・シール・真空・搬送・精密機構等の半導体製造装置内蔵部品/サブシステム（SMC等）。AI半導体増産で装置需要拡大の恩恵</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SEG016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>電子部品・パッケージ基板・産業ガス等（周辺・下流）</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>半導体周辺</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>16</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>完了</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>ICパッケージ基板・MLCC・産業/特殊ガス・前駆体材料等の周辺/下流。AIサーバー・AI半導体需要で構造的に拡大</t>
         </is>
       </c>
     </row>
@@ -10898,7 +12328,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H202"/>
+  <dimension ref="A1:H219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18553,6 +19983,720 @@
         </is>
       </c>
     </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>S217</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>C138</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>決算</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>SMC【6273】決算発表・業績情報</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>日本経済新聞</t>
+        </is>
+      </c>
+      <c r="F203" t="inlineStr">
+        <is>
+          <t>https://www.nikkei.com/nkd/company/kessan/?scode=6273</t>
+        </is>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>2026年5月14日発表; [SMC 空気圧機器グローバルトップ](https://froggy.smbcnikko.co.jp/69394/) 日興フロッギー</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>S218</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>C139</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>IR</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>IR説明会資料・決算資料</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>CKD株式会社</t>
+        </is>
+      </c>
+      <c r="F204" t="inlineStr">
+        <is>
+          <t>https://www.ckd.co.jp/ir/kessan/</t>
+        </is>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>2026年; [CKD（6407）会社業績](https://irbank.net/E01909/pl) IRBANK</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>S219</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>C140</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>決算</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>PILLAR【6490】決算発表・業績情報</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>日本経済新聞</t>
+        </is>
+      </c>
+      <c r="F205" t="inlineStr">
+        <is>
+          <t>https://www.nikkei.com/nkd/company/kessan/?scode=6490</t>
+        </is>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>2026年5月発表; [ＰＩＬＬＡＲ 業績・財務推移](https://kabutan.jp/stock/finance?code=6490) 株探</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>S220</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>C141</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>決算説明会</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>イーグル工業 決算説明会書き起こし</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>Yahoo!ファイナンス</t>
+        </is>
+      </c>
+      <c r="F206" t="inlineStr">
+        <is>
+          <t>https://finance.yahoo.co.jp/quote/6486.T/financials?styl=presentation</t>
+        </is>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>2026年; [イーグル工業 決算情報・業績](https://minkabu.jp/stock/6486/settlement) みんかぶ</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>S221</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>C142</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>決算短信</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>堀場製作所 2026年12月期 第1四半期決算・通期見通し</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>IR-tracker</t>
+        </is>
+      </c>
+      <c r="F207" t="inlineStr">
+        <is>
+          <t>https://www.ir-tracker.com/ja/articles/6856-2026-Q1</t>
+        </is>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>2026年; [6856 堀場製作所 決算発表履歴（適時開示）](https://irbank.net/6856/pl) IRBANK</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>S222</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>C143</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>企業分析</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>ローツェ 企業情報・業績（EFEM世界シェア25〜35%）</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>バフェット・コード</t>
+        </is>
+      </c>
+      <c r="F208" t="inlineStr">
+        <is>
+          <t>https://www.buffett-code.com/company/6323/</t>
+        </is>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>2026年; [企業研究！ローツェ（6323）半導体搬送のニッチトップ](https://note.com/eight4413/n/n5a8aa74b220c) note</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>S223</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>C144</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>決算短信</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>2026年3月期 決算短信〔IFRS〕(連結)</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>株式会社アドバンテスト</t>
+        </is>
+      </c>
+      <c r="F209" t="inlineStr">
+        <is>
+          <t>https://www.advantest.com/ja/news/2026/a81o6o0000000heh-att/J_FR_FY2025_FN.pdf</t>
+        </is>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>2026年4月27日</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>S224</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>C145</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>IR</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>ダイフク【6383】IR情報・決算短信</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>日本経済新聞</t>
+        </is>
+      </c>
+      <c r="F210" t="inlineStr">
+        <is>
+          <t>https://www.nikkei.com/nkd/company/kigyo/?scode=6383</t>
+        </is>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>2026年; [ダイフクは連日の上場来高値更新、収益拡大評価の買い続く](https://shikiho.toyokeizai.net/news/0/910373) 会社四季報</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>S225</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>C146</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>決算説明資料</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>2026年3月期 決算説明資料・中期経営計画骨子</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>株式会社フェローテックホールディングス</t>
+        </is>
+      </c>
+      <c r="F211" t="inlineStr">
+        <is>
+          <t>https://japanir.jp/company/company-6890/ir/6890-20260518-01_wp_financial_summary/</t>
+        </is>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>2026年5月18日</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>S226</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>C147</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>報道</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>イビデン、半導体部品増産へ5000億円投資 生成AIサーバー向け</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>日本経済新聞</t>
+        </is>
+      </c>
+      <c r="F212" t="inlineStr">
+        <is>
+          <t>https://www.nikkei.com/article/DGXZQOFD0370L0T00C26A2000000/</t>
+        </is>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>2026年2月; [イビデン26年3月期、純利益340億円 AIサーバー向け好調で一転増益](https://www.nikkei.com/article/DGXZQOFD0176E0R00C25A8000000/) 日本経済新聞</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>S227</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>C148</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>決算短信</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>決算短信 IRライブラリ</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>新光電気工業株式会社</t>
+        </is>
+      </c>
+      <c r="F213" t="inlineStr">
+        <is>
+          <t>https://www.shinko.co.jp/ir/library/summary/</t>
+        </is>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>2026年; [新光電気工業、AI半導体「後工程」の覇者へ](https://note.com/loyal_myrtle1528/n/nd95d766f62ee) note</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>S228</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>C149</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>報道</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>半年で株価3倍の村田製作所、「AIサーバー特需」は続くか</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>東洋経済オンライン</t>
+        </is>
+      </c>
+      <c r="F214" t="inlineStr">
+        <is>
+          <t>https://toyokeizai.net/articles/-/947755</t>
+        </is>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>2026年; [村田製が急騰、MLCCのAIデータセンター向け爆需獲得で業績変貌](https://kabutan.jp/news/marketnews/?b=n202605210546) 株探</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>S229</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>C150</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>決算発表</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>TDK Posts Record Profits Driven by AI Data Center Demand (FY2026 Full-Year Earnings Call)</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>BigGo Finance</t>
+        </is>
+      </c>
+      <c r="F215" t="inlineStr">
+        <is>
+          <t>https://finance.biggo.com/news/JP_6762.T_2026-04-28</t>
+        </is>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>2026年4月28日</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>S230</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>C151</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>決算</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>日本酸素ホールディングス 決算情報</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>松井証券</t>
+        </is>
+      </c>
+      <c r="F216" t="inlineStr">
+        <is>
+          <t>https://finance.matsui.co.jp/stock/4091/settlement/index</t>
+        </is>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>2026年; [日本酸素HD 業績・財務推移](https://kabutan.jp/stock/finance?code=4091) 株探</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>S231</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>C152</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>決算</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>関東電化工業 決算発表履歴（適時開示）</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>IRBANK</t>
+        </is>
+      </c>
+      <c r="F217" t="inlineStr">
+        <is>
+          <t>https://irbank.net/4047/pl</t>
+        </is>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>2026年; [関東電化工業 決算情報・業績](https://minkabu.jp/stock/4047/settlement) みんかぶ</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>S232</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>C153</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>決算分析</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>トリケミカル研究所（4369）2026年1月期3Q決算：生成AI需要で3割増益</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>note（日本株ラボ）</t>
+        </is>
+      </c>
+      <c r="F218" t="inlineStr">
+        <is>
+          <t>https://note.com/jstock_lab/n/n3d8f9723f4aa</t>
+        </is>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>2026年; [トリケミカル研究所 IR情報・中期経営計画](https://www.nikkei.com/nkd/company/kigyo/?scode=4369) 日本経済新聞</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>S233</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>C154</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>決算説明会</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>太陽誘電、営業益91％増の200億円に急回復 来期は50％増の300億円計画 AIサーバー需要追い風</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>BigGo Finance</t>
+        </is>
+      </c>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>https://finance.biggo.jp/news/JP_6976.T_2026-05-08</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>2026年5月8日</t>
+        </is>
+      </c>
+      <c r="H219" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add SEG017 (DC construction SI / DC operators) and reflect in outputs
Integrate the "build the IT inside the box → operate" layer (SEG017,
8 companies) as the flow's final step before service go-live in both
the flow HTML and deck slide 2, relabel the parts/materials/gas band
as a SUPPORT layer, add a領域07 appendix slide, and regenerate the
master xlsx (153 companies). Pure IT distributors/software SI are
documented as out-of-scope for ANDPAD targeting.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017hVm54qQ8iaGNRYcCDuKBy
</commit_message>
<xml_diff>
--- a/output/valuechain_master.xlsx
+++ b/output/valuechain_master.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P146"/>
+  <dimension ref="A1:P154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -11706,6 +11706,630 @@
         </is>
       </c>
     </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>17</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>DC・IT</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>SEG017</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>データセンター構築・ITインフラSI／DC運営</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>C157</t>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>NTTデータグループ</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr">
+        <is>
+          <t>NTT DATA Group Corporation</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>9613</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr">
+        <is>
+          <t>DCをAI時代の中核インフラと位置づけ2030年度に3ギガワット超の提供規模を目標。外部ファンドと共同出資会社を設立し今後5年でDC投資を数千億円積み増す計画でAIを成長エンジンに営業収益は初の5兆円超（発注者A：ハイパースケールDC新設を発注）。</t>
+        </is>
+      </c>
+      <c r="N147" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O147" t="inlineStr">
+        <is>
+          <t>AIを中核とした成長戦略をグローバルで加速（https://www.nttdata.com/global/ja/news/release/2026/050806/） / NTTデータ ファンドと組みデータセンター拡大 数千億円投資上積み（https://www.nikkei.com/article/DGXZQOUC197L40Z10C26A6000000/）</t>
+        </is>
+      </c>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>17</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>DC・IT</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>SEG017</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>データセンター構築・ITインフラSI／DC運営</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>C155</t>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>さくらインターネット</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr">
+        <is>
+          <t>SAKURA internet Inc.</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>3778</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr">
+        <is>
+          <t>生成AI向けGPUインフラ拡大に向け石狩DCの拡張・液冷導入を進めコンテナ型DCでNVIDIA Blackwell GPU約1100基を稼働。2026年3月期のDC設備投資は668億円規模でGPUインフラ売上は前期比+20.3%（発注者A：自社DC新設・GPU据付を発注）。</t>
+        </is>
+      </c>
+      <c r="N148" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O148" t="inlineStr">
+        <is>
+          <t>2026年3月期期末 決算説明資料（https://www.sakura.ad.jp/corporate/wp-content/uploads/2026/04/260427-ir_2.pdf） / 「NVIDIA Blackwell GPU」約1,100基を搭載したAIインフラの稼働を開始（https://www.sakura.ad.jp/corporate/information/newsreleases/2026/02/25/1968223641/）</t>
+        </is>
+      </c>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>17</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>DC・IT</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>SEG017</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>データセンター構築・ITインフラSI／DC運営</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>C156</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>インターネットイニシアティブ（IIJ）</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr">
+        <is>
+          <t>Internet Initiative Japan Inc.</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>3774</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr">
+        <is>
+          <t>自社サービス需要拡大で白井DCキャンパス3期棟（約1000ラック規模・投資額約300億円）を増設し2026年度運用開始。AI用GPUサーバーの高発熱に備え直接水冷（DLC）対応の水冷Ready設計を採用（発注者A：DC新設・水冷配管/AIサーバー据付を発注）。</t>
+        </is>
+      </c>
+      <c r="N149" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O149" t="inlineStr">
+        <is>
+          <t>IIJ 自社サービス需要拡大に対応し「白井データセンターキャンパス」3期棟を増設（https://www.iij.ad.jp/news/pressrelease/2025/0508.html）</t>
+        </is>
+      </c>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>17</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>DC・IT</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>SEG017</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>データセンター構築・ITインフラSI／DC運営</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>C160</t>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>伊藤忠テクノソリューションズ（CTC）</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr">
+        <is>
+          <t>ITOCHU Techno-Solutions Corporation</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>4739</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr">
+        <is>
+          <t>クラウド・GPU基盤サービスが牽引し2026年3月期は売上収益7937億円（+9%）・営業利益804億円（+19%）2027年3月期も増益計画。オンプレ生成AI基盤「CUVIC GPU Zero」等を展開（A＋Bハイブリッド：自社DC発注＋顧客DC/GPU基盤の構築・据付を請負）。</t>
+        </is>
+      </c>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O150" t="inlineStr">
+        <is>
+          <t>決算関連情報（IR）; CTCの27年3月期、純利益7％増の650億円 クラウド好調（https://www.ctc-g.co.jp/company/ir/）</t>
+        </is>
+      </c>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>17</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>DC・IT</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>SEG017</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>データセンター構築・ITインフラSI／DC運営</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>C159</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>兼松エレクトロニクス</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr">
+        <is>
+          <t>Kanematsu Electronics Ltd.</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>8096</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr">
+        <is>
+          <t>ネットワーク機器・生成AI関連機器の需要とDCインフラ構築需要で3期ぶり増収増益。2026年3月期は売上収益1073億円（+9.7%）・営業利益108億円（+37.2%）2027年3月期は売上1288億円（+20.0%）で過去最高益計画（請負B：サーバー/NW機器の設計・構築・据付を担うITファシリティSIer）。</t>
+        </is>
+      </c>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>高</t>
+        </is>
+      </c>
+      <c r="O151" t="inlineStr">
+        <is>
+          <t>兼松エレクトロニクス 決算情報（2026年3月期 売上収益1073億円・営業利益108億円）（https://www.nikkei.com/nkd/company/?nik_code=0022095）</t>
+        </is>
+      </c>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>17</v>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>DC・IT</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>SEG017</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
+          <t>データセンター構築・ITインフラSI／DC運営</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>C161</t>
+        </is>
+      </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>NECネッツエスアイ</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr">
+        <is>
+          <t>NEC Networks &amp; System Integration Corporation</t>
+        </is>
+      </c>
+      <c r="I152" t="inlineStr"/>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>非上場（NEC完全子会社／旧東証プライム1973・2025年3月上場廃止）</t>
+        </is>
+      </c>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr">
+        <is>
+          <t>企業のAIエージェント/AIインフラ（NW・セキュリティ・コンピューティング）の設計・構築を提供しシスコと連携しCisco AI PODs等を活用した最先端AIインフラ構築・実証を推進（請負B：NW・通信設備・DCファシリティの物理構築/据付を担うエンジニアリング系SIer）。</t>
+        </is>
+      </c>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="O152" t="inlineStr">
+        <is>
+          <t>AIエージェントの業務利用促進を目指すプロジェクトを始動（AIインフラ構築・実証）（https://www.nesic.co.jp/news/2025/20251204.html）</t>
+        </is>
+      </c>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>17</v>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>DC・IT</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>SEG017</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>データセンター構築・ITインフラSI／DC運営</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>C162</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>NTTファシリティーズ</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>NTT FACILITIES INC.</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr"/>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>非上場（NTT完全子会社）</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>生成AI時代の高発熱GPUサーバー対応のDC冷却（液冷・チラーレス液冷空調含む）の設計・施工力を強化し武蔵野に空調実機と模擬負荷（空冷420kW・液冷216kW）を備えた検証施設を構築（請負B：電源・空調・液冷設備の据付/試運転を担うDC設計施工大手）。</t>
+        </is>
+      </c>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>生成AI時代のデータセンター空調技術を結集させた検証施設（https://www.ntt-f.co.jp/news/2025/20250415.html）</t>
+        </is>
+      </c>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>17</v>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>DC・IT</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>SEG017</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>データセンター構築・ITインフラSI／DC運営</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>C158</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>アイネット</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>INET Corporation</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>9600</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>東証プライム</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>上場</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>日本</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>横浜の自社DCと連携する新DC「inet annex」を2026年1月に開所しDC・クラウド事業で増収増益を継続。生成AI・GPU需要の受け皿を拡張（発注者A：自社DC新設・増床を発注／上場廃止予定）。</t>
+        </is>
+      </c>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>新たなデータセンター「inet annex」を2026年1月に開所（https://www.inet.co.jp/news/2026/20260121.html）</t>
+        </is>
+      </c>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -11717,7 +12341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12314,6 +12938,41 @@
       <c r="G17" t="inlineStr">
         <is>
           <t>ICパッケージ基板・MLCC・産業/特殊ガス・前駆体材料等の周辺/下流。AIサーバー・AI半導体需要で構造的に拡大</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SEG017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>データセンター構築・ITインフラSI／DC運営</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>DC・IT</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>17</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>中</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>完了</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>箱（建屋）完成後にIT機器を搬入・据付・構築して稼働させる層。DC構築ITファシリティSIer（請負）と自社DCを建設するDC運営事業者（発注者）。AI/GPU基盤の物理現場工事でANDPAD現場管理と親和</t>
         </is>
       </c>
     </row>
@@ -12328,7 +12987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H219"/>
+  <dimension ref="A1:H229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20697,6 +21356,426 @@
         </is>
       </c>
     </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>S234</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>C155</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>決算説明資料</t>
+        </is>
+      </c>
+      <c r="D220" t="inlineStr">
+        <is>
+          <t>2026年3月期期末 決算説明資料</t>
+        </is>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>さくらインターネット株式会社</t>
+        </is>
+      </c>
+      <c r="F220" t="inlineStr">
+        <is>
+          <t>https://www.sakura.ad.jp/corporate/wp-content/uploads/2026/04/260427-ir_2.pdf</t>
+        </is>
+      </c>
+      <c r="G220" t="inlineStr">
+        <is>
+          <t>2026年4月27日</t>
+        </is>
+      </c>
+      <c r="H220" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>S235</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>C155</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>プレスリリース</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>「NVIDIA Blackwell GPU」約1,100基を搭載したAIインフラの稼働を開始</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>さくらインターネット株式会社</t>
+        </is>
+      </c>
+      <c r="F221" t="inlineStr">
+        <is>
+          <t>https://www.sakura.ad.jp/corporate/information/newsreleases/2026/02/25/1968223641/</t>
+        </is>
+      </c>
+      <c r="G221" t="inlineStr">
+        <is>
+          <t>2026年2月25日</t>
+        </is>
+      </c>
+      <c r="H221" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>S236</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>C156</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>プレスリリース</t>
+        </is>
+      </c>
+      <c r="D222" t="inlineStr">
+        <is>
+          <t>IIJ 自社サービス需要拡大に対応し「白井データセンターキャンパス」3期棟を増設</t>
+        </is>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>株式会社インターネットイニシアティブ</t>
+        </is>
+      </c>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>https://www.iij.ad.jp/news/pressrelease/2025/0508.html</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>2025年5月8日</t>
+        </is>
+      </c>
+      <c r="H222" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>S237</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>C157</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>プレスリリース</t>
+        </is>
+      </c>
+      <c r="D223" t="inlineStr">
+        <is>
+          <t>AIを中核とした成長戦略をグローバルで加速</t>
+        </is>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>NTTデータグループ</t>
+        </is>
+      </c>
+      <c r="F223" t="inlineStr">
+        <is>
+          <t>https://www.nttdata.com/global/ja/news/release/2026/050806/</t>
+        </is>
+      </c>
+      <c r="G223" t="inlineStr">
+        <is>
+          <t>2026年5月8日</t>
+        </is>
+      </c>
+      <c r="H223" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>S238</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>C157</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>報道</t>
+        </is>
+      </c>
+      <c r="D224" t="inlineStr">
+        <is>
+          <t>NTTデータ ファンドと組みデータセンター拡大 数千億円投資上積み</t>
+        </is>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>日本経済新聞</t>
+        </is>
+      </c>
+      <c r="F224" t="inlineStr">
+        <is>
+          <t>https://www.nikkei.com/article/DGXZQOUC197L40Z10C26A6000000/</t>
+        </is>
+      </c>
+      <c r="G224" t="inlineStr">
+        <is>
+          <t>2026年6月</t>
+        </is>
+      </c>
+      <c r="H224" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>S239</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>C158</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>プレスリリース</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>新たなデータセンター「inet annex」を2026年1月に開所</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>株式会社アイネット</t>
+        </is>
+      </c>
+      <c r="F225" t="inlineStr">
+        <is>
+          <t>https://www.inet.co.jp/news/2026/20260121.html</t>
+        </is>
+      </c>
+      <c r="G225" t="inlineStr">
+        <is>
+          <t>2026年1月21日</t>
+        </is>
+      </c>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>S240</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>C159</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>決算</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>兼松エレクトロニクス 決算情報（2026年3月期 売上収益1073億円・営業利益108億円）</t>
+        </is>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>日本経済新聞（決算短信に基づく）</t>
+        </is>
+      </c>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>https://www.nikkei.com/nkd/company/?nik_code=0022095</t>
+        </is>
+      </c>
+      <c r="G226" t="inlineStr">
+        <is>
+          <t>2026年5月</t>
+        </is>
+      </c>
+      <c r="H226" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>S241</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>C160</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>IR</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>決算関連情報（IR）; CTCの27年3月期、純利益7％増の650億円 クラウド好調</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>CTC 伊藤忠テクノソリューションズ／日本経済新聞</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>https://www.ctc-g.co.jp/company/ir/</t>
+        </is>
+      </c>
+      <c r="G227" t="inlineStr">
+        <is>
+          <t>2026年5月</t>
+        </is>
+      </c>
+      <c r="H227" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>S242</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>C161</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>プレスリリース</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>AIエージェントの業務利用促進を目指すプロジェクトを始動（AIインフラ構築・実証）</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>NECネッツエスアイ株式会社</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>https://www.nesic.co.jp/news/2025/20251204.html</t>
+        </is>
+      </c>
+      <c r="G228" t="inlineStr">
+        <is>
+          <t>2025年12月4日</t>
+        </is>
+      </c>
+      <c r="H228" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>S243</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>C162</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>プレスリリース</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>生成AI時代のデータセンター空調技術を結集させた検証施設</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>株式会社NTTファシリティーズ</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>https://www.ntt-f.co.jp/news/2025/20250415.html</t>
+        </is>
+      </c>
+      <c r="G229" t="inlineStr">
+        <is>
+          <t>2025年4月15日</t>
+        </is>
+      </c>
+      <c r="H229" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>